<commit_message>
MarineBoard v1.9: RGB status LED, vertical CN4 display header, logo, fab package (#179)
- D17 plain LED -> D5 WS2812B-2020-V6 (C52917434) on GPIO1, VDD +5V_VCC,
  C40 decoupling, R34 100R on DIN
- U10 right-angle GH on the bottom -> CN4 vertical BM10B-GHS-TBT on top
  (pinout unchanged); all fuses/connectors on top; GND stitching reworked
- Sisu logo + "MARINE BOARD v1.9" silk (LOGO1), RESET/FLASH labels
- Libraries consolidated back into Lib/ (root EasyEDA.* retired), CN4
  courtyard now covers its leads, L2 footprint attr THT -> SMD
- fab_package.py rebuilds production/ (DRC gate, gerbers/drill/IPC zip,
  BOM + centroid CSV/XLSX with LOOSE rows); stale production files removed
- Technical Specs v1.9 (CN4, RGB LED, fab script, U5/U6/U7 pin order),
  system spec 2.15, README, feature map, HEADER PINS / LEDS exports

Firmware follow-up for the RGB LED: #180

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MarineBoard/production/MarineBoard-BOM.xlsx
+++ b/MarineBoard/production/MarineBoard-BOM.xlsx
@@ -27,20 +27,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,9 +51,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -510,7 +502,6 @@
       <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>KLJ-4020</t>
@@ -541,7 +532,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -555,7 +545,6 @@
       <c r="C3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>CL05A106MQ5NUNC</t>
@@ -586,7 +575,6 @@
           <t>Bottom/Top</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -594,13 +582,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C2,C3,C5,C7,C9,C11,C12,C14,C19,C22,C24,C27,C28,C31,C32,C34,C35,C36,C37,C38,C42</t>
+          <t>C2,C3,C5,C7,C9,C11,C12,C14,C19,C22,C24,C27,C28,C31,C32,C34,C35,C36,C37,C38,C40,C42</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>22</v>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>CL05B104KO5NNNC</t>
@@ -631,7 +618,6 @@
           <t>Bottom/Top</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -645,7 +631,6 @@
       <c r="C5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>C3845593</t>
@@ -676,7 +661,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -690,7 +674,6 @@
       <c r="C6" t="n">
         <v>1</v>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>C88896</t>
@@ -721,7 +704,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -735,7 +717,6 @@
       <c r="C7" t="n">
         <v>3</v>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>CL05A475MP5NRNC</t>
@@ -766,7 +747,6 @@
           <t>Bottom/Top</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -780,7 +760,6 @@
       <c r="C8" t="n">
         <v>1</v>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>GRM21BR61H106KE43L</t>
@@ -811,7 +790,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -825,7 +803,6 @@
       <c r="C9" t="n">
         <v>1</v>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>GRM31CR61E476ME44L</t>
@@ -856,7 +833,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -870,7 +846,6 @@
       <c r="C10" t="n">
         <v>1</v>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>C51205</t>
@@ -901,7 +876,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -915,7 +889,6 @@
       <c r="C11" t="n">
         <v>1</v>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>C13585</t>
@@ -946,7 +919,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -960,7 +932,6 @@
       <c r="C12" t="n">
         <v>1</v>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>CL05B103KB5NNNC</t>
@@ -991,7 +962,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1005,7 +975,6 @@
       <c r="C13" t="n">
         <v>1</v>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>C72494</t>
@@ -1036,7 +1005,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1050,7 +1018,6 @@
       <c r="C14" t="n">
         <v>1</v>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>GRM1555C1H152JA01D</t>
@@ -1081,7 +1048,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1095,7 +1061,6 @@
       <c r="C15" t="n">
         <v>1</v>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>GRM1555C1H151JA01D</t>
@@ -1126,7 +1091,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1140,7 +1104,6 @@
       <c r="C16" t="n">
         <v>2</v>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>GCM155R71H473KE02D</t>
@@ -1171,7 +1134,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1185,7 +1147,6 @@
       <c r="C17" t="n">
         <v>1</v>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>C37323734</t>
@@ -1216,7 +1177,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1230,7 +1190,6 @@
       <c r="C18" t="n">
         <v>2</v>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>1729128</t>
@@ -1261,7 +1220,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1275,7 +1233,6 @@
       <c r="C19" t="n">
         <v>1</v>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>SM04B-SRSS-TB(LF)(SN)</t>
@@ -1306,7 +1263,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1314,31 +1270,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>D1,D4,D15</t>
+          <t>CN4</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
-      </c>
-      <c r="D20" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SS14</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>40V 1A Schottky Diode, SMA</t>
+          <t>BM10B-GHS-TBT(LF)(SN)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>SS14</t>
+          <t>BM10B-GHS-TBT</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>D_SMA</t>
+          <t>CONN-SMD_BM10B-GHS-TBT-LF-SN</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1348,10 +1298,9 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1359,35 +1308,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>D2,D3</t>
+          <t>D1,D4,D15</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>R+O(宏嘉诚)</t>
-        </is>
+        <v>3</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>C7420372</t>
+          <t>SS14</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>极性:双向;反向截止电压(Vrwm):5V;钳位电压:10V;峰值脉冲电流(Ipp):5A;峰值脉冲功率(Ppp):50W;击穿电压:5.6V;</t>
+          <t>40V 1A Schottky Diode, SMA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>H5VL10B</t>
+          <t>SS14</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>D_SOD-882</t>
+          <t>D_SMA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1397,10 +1341,9 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
+          <t>Bottom/Top</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1408,31 +1351,35 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D2,D3</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>R+O(宏嘉诚)</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SMBJ18A</t>
+          <t>C7420372</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>29.2VC Clamp 20.6A@10/1000us Ipp TVS DIODE DO-214AA(SMB)</t>
+          <t>极性:双向;反向截止电压(Vrwm):5V;钳位电压:10V;峰值脉冲电流(Ipp):5A;峰值脉冲功率(Ppp):50W;击穿电压:5.6V;</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SMBJ18A</t>
+          <t>H5VL10B</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>D_SMB</t>
+          <t>D_SOD-882</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1445,7 +1392,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1453,27 +1399,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>1</v>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>C417538</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>C52917434</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>RGB LED with integrated controller, 2.0 x 2.0 mm, 12 mA</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>LMBR340FT1G</t>
+          <t>WS2812B-2020</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>D_SOD-123F</t>
+          <t>LED_WS2812B-2020_PLCC4_2.0x2.0mm</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1486,7 +1435,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1494,27 +1442,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>1</v>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>C506523</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>SMBJ18A</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>29.2VC Clamp 20.6A@10/1000us Ipp TVS DIODE DO-214AA(SMB)</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>VS-43CTQ100S-M3</t>
+          <t>SMBJ18A</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>D2PAK_L10.0-W9.0-P2.54-LS15.0-TL-1</t>
+          <t>D_SMB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1524,10 +1475,9 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1535,31 +1485,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>D9,D11,D12,D13,D18,D19</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6</v>
-      </c>
-      <c r="D25" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ESD5Z3.3T1G</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>14VC Clamp 11A Ipp ESD DIODE SOD-523</t>
+          <t>C417538</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ESD5Z3.3T1G</t>
+          <t>LMBR340FT1G</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>D_SOD-523</t>
+          <t>D_SOD-123F</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1569,10 +1513,9 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1580,27 +1523,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>1</v>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>C2687121</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>C506523</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>PESD1CAN</t>
+          <t>VS-43CTQ100S-M3</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>D2PAK_L10.0-W9.0-P2.54-LS15.0-TL-1</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1613,7 +1554,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1621,27 +1561,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D9,D11,D12,D13,D18,D19</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" t="inlineStr"/>
+        <v>6</v>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>C18199169</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>ESD5Z3.3T1G</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>14VC Clamp 11A Ipp ESD DIODE SOD-523</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>SS56</t>
+          <t>ESD5Z3.3T1G</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>D_SMA</t>
+          <t>D_SOD-523</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1651,10 +1594,9 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
+          <t>Bottom/Top</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1662,31 +1604,25 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>D16,D17</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>C2286</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Light emitting diode</t>
+          <t>C2687121</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>LED</t>
+          <t>PESD1CAN</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>LED_0603_1608Metric</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1699,7 +1635,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1707,31 +1642,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>1</v>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>C12790</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>MBRS3100T3G</t>
+          <t>C18199169</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MBRS3100T3G</t>
+          <t>SS56</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>D_SMC</t>
+          <t>D_SMA</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1744,7 +1673,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1752,27 +1680,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>1</v>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>C70426</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>C2286</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Light emitting diode</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>S3MB-13-F</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>D_SMB</t>
+          <t>LED_0603_1608Metric</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1785,7 +1716,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1793,40 +1723,42 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>1</v>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>C492610</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+          <t>C12790</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>MBRS3100T3G</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>MBRS3100T3G</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>FUSE-TH_XF-506P</t>
+          <t>D_SMC</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1834,40 +1766,37 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>1</v>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>C492610</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>C70426</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>S3MB-13-F</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>FUSE-TH_XF-506P</t>
+          <t>D_SMB</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1875,22 +1804,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>F3,F4</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
-      </c>
-      <c r="D33" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>C492610</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1908,7 +1835,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1916,36 +1842,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Flash1</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>1</v>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>C318884</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Push button switch, generic, two pins</t>
+          <t>C492610</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Flash</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>SW_Push_1P1T_XKB_TS-1187A</t>
+          <t>FUSE-TH_XF-506P</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -1953,7 +1873,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1961,36 +1880,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>F3,F4</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>C2894897</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>USB 2.0-only 16P Type-C Receptacle connector</t>
+          <t>C492610</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>USB_C_Receptacle_USB2.0_16P</t>
+          <t>10A</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>USB_C_Receptacle_HCTL_HC-TYPE-C-16P-01A</t>
+          <t>FUSE-TH_XF-506P</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -1998,7 +1911,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2006,42 +1918,40 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JP1</t>
+          <t>Flash1</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>1</v>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>C703015</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>C318884</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Push button switch, generic, two pins</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>CAN Bus Term</t>
+          <t>Flash</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>PinHeader_1x02_P1.27mm_Vertical</t>
+          <t>SW_Push_1P1T_XKB_TS-1187A</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
           <t>Top</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Leave open - supply shunt loose</t>
         </is>
       </c>
     </row>
@@ -2051,27 +1961,30 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C37" t="n">
         <v>1</v>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>C435392</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>C2894897</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>USB 2.0-only 16P Type-C Receptacle connector</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>1uH 3.3A 40mΩ</t>
+          <t>USB_C_Receptacle_USB2.0_16P</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>L_1008_2520Metric</t>
+          <t>USB_C_Receptacle_HCTL_HC-TYPE-C-16P-01A</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2084,7 +1997,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2092,27 +2004,25 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>JP1</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>1</v>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>C5368704</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>C703015</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>22uH</t>
+          <t>CAN Bus Term</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>IND-SMD_L12.5-W12.5_B82477P4XX</t>
+          <t>PinHeader_1x02_P1.27mm_Vertical</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2122,10 +2032,14 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Leave open - supply shunt loose</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2133,35 +2047,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>L3,L4,L6</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>muRata(村田)</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>C79382</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>标称阻抗@测试频率:120Ω@100MHz;误差:±25%;直流电阻(RDC):30mΩ;</t>
+          <t>C435392</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>BLM21PG121SN1D</t>
+          <t>1uH 3.3A 40mΩ</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>L_0805_2012Metric</t>
+          <t>L_1008_2520Metric</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2171,10 +2075,9 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2182,27 +2085,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C40" t="n">
         <v>1</v>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>C225048</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>C5368704</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>CDRH104RNP-150NC</t>
+          <t>22uH</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>IND-SMD_L10.2-W10.0</t>
+          <t>IND-SMD_L12.5-W12.5_B82477P4XX</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2212,10 +2113,9 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2223,22 +2123,30 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>L7,L9,L10</t>
+          <t>L3,L4,L6</t>
         </is>
       </c>
       <c r="C41" t="n">
         <v>3</v>
       </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>muRata(村田)</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>C74764</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>C79382</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>标称阻抗@测试频率:120Ω@100MHz;误差:±25%;直流电阻(RDC):30mΩ;</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>FerriteBead</t>
+          <t>BLM21PG121SN1D</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2253,10 +2161,9 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr"/>
+          <t>Bottom/Top</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2264,27 +2171,25 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>L8</t>
+          <t>L5</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>1</v>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>C97856</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>C225048</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>DLW21SN900SQ2L</t>
+          <t>CDRH104RNP-150NC</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>FILTER-SMD_4P-L2.0-W1.2-BL_DLW21H</t>
+          <t>IND-SMD_L10.2-W10.0</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2294,10 +2199,9 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2305,35 +2209,25 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Q2,Q3</t>
+          <t>L7,L9,L10</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>宏嘉诚</t>
-        </is>
+        <v>3</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>C20069125</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>晶体管类型:NPN;集电极电流(Ic):500mA;集射极击穿电压(Vceo):25V;耗散功率(Pd):300mW;直流电流增益(hFE):120@50mA,1.0V;</t>
+          <t>C74764</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>S8050</t>
+          <t>FerriteBead</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>L_0805_2012Metric</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2346,7 +2240,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2354,27 +2247,25 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>L8</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>1</v>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>C52191006</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
+          <t>C97856</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>BUK762R4-60E</t>
+          <t>DLW21SN900SQ2L</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TO-263-2_L10.1-W9.1-P5.08-LS15.2-BR</t>
+          <t>FILTER-SMD_4P-L2.0-W1.2-BL_DLW21H</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2384,10 +2275,9 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2395,31 +2285,35 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>R1,R2</t>
+          <t>Q2,Q3</t>
         </is>
       </c>
       <c r="C45" t="n">
         <v>2</v>
       </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>宏嘉诚</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C20069125</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>晶体管类型:NPN;集电极电流(Ic):500mA;集射极击穿电压(Vceo):25V;耗散功率(Pd):300mW;直流电流增益(hFE):120@50mA,1.0V;</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>5.1K</t>
+          <t>S8050</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2432,7 +2326,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2440,31 +2333,25 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>R3,R10,R15,R20,R25,R26,R27,R28,R32,R40,R42,R43</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>12</v>
-      </c>
-      <c r="D46" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>C25744</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C52191006</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>BUK762R4-60E</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>TO-263-2_L10.1-W9.1-P5.08-LS15.2-BR</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2474,10 +2361,9 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2485,27 +2371,30 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R1,R2</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>C149504</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>C25905</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Resistor</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>100K</t>
+          <t>5.1K</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2515,10 +2404,9 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2526,16 +2414,15 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>R5,R6</t>
+          <t>R3,R10,R15,R20,R25,R26,R27,R28,R32,R40,R42,R43</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" t="inlineStr"/>
+        <v>12</v>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>C25105</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2545,7 +2432,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>33R</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2560,10 +2447,9 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr"/>
+          <t>Bottom/Top</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2571,22 +2457,20 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>R7,R9,R35,R36</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
-      </c>
-      <c r="D49" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>C2907296</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>C149504</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100K</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2601,10 +2485,9 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2612,31 +2495,30 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R5,R6</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>C17560</t>
+          <t>C25105</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>22KΩ (2202) ±1%</t>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>22K</t>
+          <t>33R</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2646,10 +2528,9 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2657,27 +2538,25 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R7,R9,R35,R36</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>C2089436</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>C2907296</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>200m</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>R_0201_0603Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2690,7 +2569,6 @@
           <t>Bottom</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2698,27 +2576,30 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="C52" t="n">
         <v>1</v>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>C53159429</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
+          <t>C17560</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>22KΩ (2202) ±1%</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>3k24</t>
+          <t>22K</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2731,7 +2612,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2739,27 +2619,25 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>1</v>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>C23079</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
+          <t>C2089436</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>549</t>
+          <t>200m</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_0201_0603Metric</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2769,10 +2647,9 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2780,27 +2657,25 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>R14,R19,R21,R23,R24,R49,R50</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>7</v>
-      </c>
-      <c r="D54" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>C17437</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
+          <t>C53159429</t>
+        </is>
+      </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>3k24</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2810,10 +2685,9 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2821,27 +2695,25 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="C55" t="n">
         <v>1</v>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>C25718</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
+          <t>C23079</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10K/1W</t>
+          <t>549</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2854,7 +2726,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2862,31 +2733,25 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>R22,R29,R30,R41,R44</t>
+          <t>R14,R19,R21,R23,R24,R49,R50</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>5</v>
-      </c>
-      <c r="D56" t="inlineStr"/>
+        <v>7</v>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>C11702</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C17437</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2899,7 +2764,6 @@
           <t>Bottom/Top</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2907,27 +2771,25 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>R31</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>1</v>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>C17408</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
+          <t>C25718</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>10K/1W</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2940,7 +2802,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2948,16 +2809,15 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>R33,R34</t>
+          <t>R22,R29,R30,R41,R44</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
-      </c>
-      <c r="D58" t="inlineStr"/>
+        <v>5</v>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>C25117</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2967,7 +2827,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>470R</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2982,10 +2842,9 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr"/>
+          <t>Bottom/Top</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2993,22 +2852,20 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>R38,R39</t>
+          <t>R31</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>C48996903</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>C17408</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3023,10 +2880,9 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3034,27 +2890,30 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>R46</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="C60" t="n">
         <v>1</v>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>C175364</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
+          <t>C25117</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Resistor</t>
+        </is>
+      </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>47K/1W</t>
+          <t>470R</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3067,7 +2926,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3075,27 +2933,30 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>R47</t>
+          <t>R34</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>1</v>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>C2075262</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
+          <t>0402WGF1000TCE</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>100Ω (1000) ±1%</t>
+        </is>
+      </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2K2</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R0402</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3105,10 +2966,9 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3116,31 +2976,25 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>R38,R39</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>C25792</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C48996903</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>47K</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3150,10 +3004,9 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3161,32 +3014,30 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Relay1</t>
+          <t>R46</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>1</v>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>C30431</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
+          <t>C175364</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>SRD-12VDC-SL-C</t>
+          <t>47K/1W</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>RELAY-TH_SRD-XXVDC-XL-C</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3194,7 +3045,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3202,31 +3052,25 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Reset1</t>
+          <t>R47</t>
         </is>
       </c>
       <c r="C64" t="n">
         <v>1</v>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>C318884</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Push button switch, generic, two pins</t>
+          <t>C2075262</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Reset</t>
+          <t>2K2</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>SW_Push_1P1T_XKB_TS-1187A</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3236,10 +3080,9 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr"/>
+          <t>Bottom</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3247,27 +3090,30 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R48</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>1</v>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>C479074</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>C25792</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Resistor</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>SY8089A1AAC</t>
+          <t>47K</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>TSOT-23-5</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3280,7 +3126,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3288,36 +3133,30 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>U2,U18,U19</t>
+          <t>Relay1</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
-      </c>
-      <c r="D66" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>INA226AQDGSRQ1</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>High-Side or Low-Side Measurement, Bi-Directional Current and Power Monitor (0-36V) with I2C Compatible Interface, VSSOP-10</t>
+          <t>C30431</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>INA226</t>
+          <t>SRD-12VDC-SL-C</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>VSSOP-10_3x3mm_P0.5mm</t>
+          <t>RELAY-TH_SRD-XXVDC-XL-C</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3325,7 +3164,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3333,31 +3171,30 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>Reset1</t>
         </is>
       </c>
       <c r="C67" t="n">
         <v>1</v>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>C502477</t>
+          <t>C318884</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>3A, Step Down Swift Converter, Adjustable Output Voltage, 5.5-36V Input Voltage, PowerSO-8</t>
+          <t>Push button switch, generic, two pins</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>TPS5430DDA</t>
+          <t>Reset</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>TI_SO-PowerPAD-8_ThermalVias</t>
+          <t>SW_Push_1P1T_XKB_TS-1187A</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3370,7 +3207,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3378,32 +3214,30 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>U4,U5,U6</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
-      </c>
-      <c r="D68" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>C466970</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
+          <t>C479074</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>DB125-3.5-2P-GN-S</t>
+          <t>SY8089A1AAC</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>CONN-TH_2P-P3.50_L7.4-W7.0</t>
+          <t>TSOT-23-5</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3411,7 +3245,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3419,32 +3252,35 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>U7,U9,U12,U13</t>
+          <t>U2,U18,U19</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>4</v>
-      </c>
-      <c r="D69" t="inlineStr"/>
+        <v>3</v>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>C466971</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
+          <t>INA226AQDGSRQ1</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>High-Side or Low-Side Measurement, Bi-Directional Current and Power Monitor (0-36V) with I2C Compatible Interface, VSSOP-10</t>
+        </is>
+      </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>DB125-3.5-3P-GN-S</t>
+          <t>INA226</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>CONN-TH_3P-P3.50_L7.4-W10.5</t>
+          <t>VSSOP-10_3x3mm_P0.5mm</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3452,7 +3288,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3460,31 +3295,30 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="C70" t="n">
         <v>1</v>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>C42417293</t>
+          <t>C502477</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2.4 GHz WiFi (802.11 b/g/n) and Bluetooth ® 5 (LE) module Built around ESP32S3 series of SoCs, Xtensa ® dualcore 32bit LX7 microprocessor Flash up to 16 MB, PSRAM up to 8 MB 36 GPIOs, rich set of peripherals Onboard PCB antenna</t>
+          <t>3A, Step Down Swift Converter, Adjustable Output Voltage, 5.5-36V Input Voltage, PowerSO-8</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-2-N32R16V</t>
+          <t>TPS5430DDA</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-2</t>
+          <t>TI_SO-PowerPAD-8_ThermalVias</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3497,7 +3331,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3505,40 +3338,37 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U4,U5,U6</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
-      </c>
-      <c r="D71" t="inlineStr"/>
+        <v>3</v>
+      </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>SM10B-GHS-TB</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
+          <t>C466970</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>SM10B-GHS-TB</t>
+          <t>DB125-3.5-2P-GN-S</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>CONN-SMD_SM10B-GHS-TB</t>
+          <t>CONN-TH_2P-P3.50_L7.4-W7.0</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3546,32 +3376,30 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U7,U9,U12,U13</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
-      </c>
-      <c r="D72" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>C12084</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
+          <t>C466971</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>SN65HVD230DR</t>
+          <t>DB125-3.5-3P-GN-S</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>CONN-TH_3P-P3.50_L7.4-W10.5</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3579,7 +3407,6 @@
           <t>Top</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3587,27 +3414,30 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>U14,U16,U17,U21</t>
+          <t>U8</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4</v>
-      </c>
-      <c r="D73" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>C3008369</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
+          <t>C42417293</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2.4 GHz WiFi (802.11 b/g/n) and Bluetooth ® 5 (LE) module Built around ESP32S3 series of SoCs, Xtensa ® dualcore 32bit LX7 microprocessor Flash up to 16 MB, PSRAM up to 8 MB 36 GPIOs, rich set of peripherals Onboard PCB antenna</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>PC817C-S</t>
+          <t>ESP32-S3-WROOM-2-N32R16V</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>SOP-4_L6.5-W4.6-P2.54-LS10.3-TL</t>
+          <t>ESP32-S3-WROOM-2</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3617,10 +3447,9 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3628,27 +3457,25 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>U22</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>1</v>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>C7835</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
+          <t>C12084</t>
+        </is>
+      </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>SN74LVC1G14DBVR</t>
+          <t>SN65HVD230DR</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3658,10 +3485,9 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr"/>
+          <t>Top</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3669,27 +3495,25 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>U23</t>
+          <t>U14,U16,U17,U21</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
-      </c>
-      <c r="D75" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>C640313</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr"/>
+          <t>C3008369</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>MCP1407-E/MF_C640313</t>
+          <t>PC817C-S</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>DFN-8_L6.0-W5.0-P1.27-BL-EP4.0</t>
+          <t>SOP-4_L6.5-W4.6-P2.54-LS10.3-TL</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3699,10 +3523,9 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr"/>
+          <t>Bottom/Top</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3710,42 +3533,35 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>F1-FUSE</t>
+          <t>U22</t>
         </is>
       </c>
       <c r="C76" t="n">
         <v>1</v>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Littelfuse</t>
-        </is>
-      </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>0297002.WXNV</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>LOOSE - MINI blade fuse 2A 32V for holder F1 (XF-506P)</t>
+          <t>C7835</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2A</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr"/>
+          <t>SN74LVC1G14DBVR</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>SOT-23-5</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>LOOSE</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>Supply loose - do NOT mount</t>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -3755,42 +3571,35 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>F2-FUSE</t>
+          <t>U23</t>
         </is>
       </c>
       <c r="C77" t="n">
         <v>1</v>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Littelfuse</t>
-        </is>
-      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>0297001.WXNV</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>LOOSE - MINI blade fuse 1A 32V for holder F2 (XF-506P)</t>
+          <t>C640313</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>1A</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr"/>
+          <t>MCP1407-E/MF_C640313</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>DFN-8_L6.0-W5.0-P1.27-BL-EP4.0</t>
+        </is>
+      </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>LOOSE</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>Supply loose - do NOT mount</t>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -3800,11 +3609,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>F3-FUSE,F4-FUSE</t>
+          <t>F1-FUSE</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3813,26 +3622,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0297010.WXNV</t>
+          <t>0297002.WXNV</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>LOOSE - MINI blade fuse 10A 32V for holders F3, F4 (XF-506P)</t>
+          <t>LOOSE - MINI blade fuse 2A 32V for holder F1 (XF-506P)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>10A</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr"/>
+          <t>2A</t>
+        </is>
+      </c>
       <c r="I78" t="inlineStr">
         <is>
           <t>LOOSE</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
           <t>Supply loose - do NOT mount</t>
@@ -3845,32 +3652,114 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
+          <t>F2-FUSE</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Littelfuse</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>0297001.WXNV</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>LOOSE - MINI blade fuse 1A 32V for holder F2 (XF-506P)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>LOOSE</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Supply loose - do NOT mount</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>F3-FUSE,F4-FUSE</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Littelfuse</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0297010.WXNV</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>LOOSE - MINI blade fuse 10A 32V for holders F3, F4 (XF-506P)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>LOOSE</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Supply loose - do NOT mount</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>JP1-SHUNT</t>
         </is>
       </c>
-      <c r="C79" t="n">
-        <v>1</v>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr">
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="inlineStr">
         <is>
           <t>LOOSE - 2-pin 1.27 mm pitch jumper shunt for JP1 (CAN termination; leave JP1 open)</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>Jumper 1.27mm</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr">
+      <c r="I81" t="inlineStr">
         <is>
           <t>LOOSE</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr">
+      <c r="K81" t="inlineStr">
         <is>
           <t>Supply loose - do NOT mount</t>
         </is>

</xml_diff>

<commit_message>
MarineBoard v1.9.1 pre-fab fixes: U3 ENA float, 50V caps, polymer C20 (#183)
- U3 TPS5430 ENA (pin 5) disconnected from VIN_BUCK (7 V abs max) and left
  floating per TI; schematic wires + PCB stub removed, no-connect added.
- C11/C12/C14/C19/C42 -> CL05B104KB5NNNC (50 V; were 16 V on 12 V/bus nets),
  C33 -> 1 uF 50 V GRM155R61H105KE05D (was 4.7 uF 10 V on +12V BAT).
- C20 -> Panasonic 10SVPE220M 20 mOhm polymer: 15 uH + 220 uF <=40 mOhm is
  TI's internal-compensation reference; the copied ceramic-cap network
  C21/C22/R13/C23 (TI Fig 7-11, 3.3 V/100 uF design) is now DNP.
- Order sheet File Name -> MarineBoard-PCBWay-Gerbers.zip.
- Fab package rebuilt; DRC (schematic parity) and ERC unchanged vs before.

Still open in #183 (routing, human): U2 VBUS, U23 supply rail, C15, D5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MarineBoard/production/MarineBoard-BOM.xlsx
+++ b/MarineBoard/production/MarineBoard-BOM.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -582,11 +582,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C2,C3,C5,C7,C9,C11,C12,C14,C19,C22,C24,C27,C28,C31,C32,C34,C35,C36,C37,C38,C40,C42</t>
+          <t>C2,C3,C5,C7,C9,C24,C27,C28,C31,C32,C34,C35,C36,C37,C38,C40</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>100nF ±10% 50V Ceramic Capacitor X7R 0402,Unpolarized capacitor</t>
+          <t>Unpolarized capacitor</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -711,11 +711,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C10,C30,C33</t>
+          <t>C10,C30</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -754,30 +754,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C11,C12,C14,C19,C42</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GRM21BR61H106KE43L</t>
+          <t>CL05B104KB5NNNC</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>10uF ±10% 50V Ceramic Capacitor X5R 0805</t>
+          <t>100nF ±10% 50V Ceramic Capacitor X7R 0402</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10uF/50V</t>
+          <t>0.1uF</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>C_0805_2012Metric</t>
+          <t>C_0402_1005Metric</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -805,22 +805,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GRM31CR61E476ME44L</t>
+          <t>GRM21BR61H106KE43L</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>47uF ±20% 25V Ceramic Capacitor X5R 1206</t>
+          <t>10uF ±10% 50V Ceramic Capacitor X5R 0805</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>47uF</t>
+          <t>10uF/50V</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>C_1206_3216Metric</t>
+          <t>C_0805_2012Metric</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -848,17 +848,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>C51205</t>
+          <t>GRM31CR61E476ME44L</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4.7uF ±10% 50V Ceramic Capacitor X7R 1206</t>
+          <t>47uF ±20% 25V Ceramic Capacitor X5R 1206</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4.7uF</t>
+          <t>47uF</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -891,17 +891,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>C13585</t>
+          <t>C51205</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10uF ±10% 50V Ceramic Capacitor X5R 1206</t>
+          <t>4.7uF ±10% 50V Ceramic Capacitor X7R 1206</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>10uF</t>
+          <t>4.7uF</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -934,22 +934,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CL05B103KB5NNNC</t>
+          <t>C13585</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10nF ±10% 50V Ceramic Capacitor X7R 0402</t>
+          <t>10uF ±10% 50V Ceramic Capacitor X5R 1206</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>10uF</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>C_0402_1005Metric</t>
+          <t>C_1206_3216Metric</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -977,22 +977,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>C72494</t>
+          <t>CL05B103KB5NNNC</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>220uF ±20% 10V Aluminum Electrolytic Capacitor 6.3x5.4mm</t>
+          <t>10nF ±10% 50V Ceramic Capacitor X7R 0402</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>220uF 10V</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CAP-SMD_BD6.3-L6.6-W6.6-FD</t>
+          <t>C_0402_1005Metric</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C21</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1020,22 +1020,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GRM1555C1H152JA01D</t>
+          <t>10SVPE220M</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.5nF ±5% 50V Ceramic Capacitor C0G 0402</t>
+          <t>220uF ±20% 10V OS-CON polymer, ESR 20mΩ, SMD D6.3xL5.9mm (TPS5430 internal comp needs ESR &lt;=40mΩ)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1.5nF</t>
+          <t>220uF 10V</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>C_0402_1005Metric</t>
+          <t>CAP-SMD_BD6.3-L6.6-W6.6-FD</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1055,25 +1055,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>C26,C29</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GRM1555C1H151JA01D</t>
+          <t>GCM155R71H473KE02D</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>150pF ±5% 50V Ceramic Capacitor C0G 0402</t>
+          <t>47nF ±10% 50V Ceramic Capacitor X7R 0402</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>150pF</t>
+          <t>47nF</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -1098,25 +1098,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C26,C29</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GCM155R71H473KE02D</t>
+          <t>GRM155R61H105KE05D</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>47nF ±10% 50V Ceramic Capacitor X7R 0402</t>
+          <t>1uF ±10% 50V Ceramic Capacitor X5R 0402</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>47nF</t>
+          <t>1uF</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2695,25 +2695,25 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R14,R19,R21,R23,R24,R49,R50</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>C23079</t>
+          <t>C17437</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>549</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -2733,25 +2733,25 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>R14,R19,R21,R23,R24,R49,R50</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>C17437</t>
+          <t>C25718</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>10K/1W</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2771,25 +2771,30 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R22,R29,R30,R41,R44</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>C25718</t>
+          <t>C11702</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>10K/1W</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2799,7 +2804,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -2809,30 +2814,25 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>R22,R29,R30,R41,R44</t>
+          <t>R31</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>C11702</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C17408</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>R31</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -2860,17 +2860,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>C17408</t>
+          <t>C25117</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>470R</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -2890,7 +2895,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>R33</t>
+          <t>R34</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -2898,22 +2903,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>C25117</t>
+          <t>0402WGF1000TCE</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>100Ω (1000) ±1%</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>470R</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R0402</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -2933,30 +2938,25 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R38,R39</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>0402WGF1000TCE</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>100Ω (1000) ±1%</t>
+          <t>C48996903</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -2976,25 +2976,25 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>R38,R39</t>
+          <t>R46</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>C48996903</t>
+          <t>C175364</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>47K/1W</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>R46</t>
+          <t>R47</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -3022,12 +3022,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>C175364</t>
+          <t>C2075262</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>47K/1W</t>
+          <t>2K2</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>R47</t>
+          <t>R48</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -3060,17 +3060,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>C2075262</t>
+          <t>C25792</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2K2</t>
+          <t>47K</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3080,7 +3085,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3095,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>Relay1</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -3098,27 +3103,22 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>C25792</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C30431</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>47K</t>
+          <t>SRD-12VDC-SL-C</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>RELAY-TH_SRD-XXVDC-XL-C</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Relay1</t>
+          <t>Reset1</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -3141,22 +3141,27 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>C30431</t>
+          <t>C318884</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Push button switch, generic, two pins</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>SRD-12VDC-SL-C</t>
+          <t>Reset</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>RELAY-TH_SRD-XXVDC-XL-C</t>
+          <t>SW_Push_1P1T_XKB_TS-1187A</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3171,7 +3176,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Reset1</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -3179,22 +3184,17 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>C318884</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Push button switch, generic, two pins</t>
+          <t>C479074</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Reset</t>
+          <t>SY8089A1AAC</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>SW_Push_1P1T_XKB_TS-1187A</t>
+          <t>TSOT-23-5</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3214,25 +3214,30 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U2,U18,U19</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>C479074</t>
+          <t>INA226AQDGSRQ1</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>High-Side or Low-Side Measurement, Bi-Directional Current and Power Monitor (0-36V) with I2C Compatible Interface, VSSOP-10</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>SY8089A1AAC</t>
+          <t>INA226</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>TSOT-23-5</t>
+          <t>VSSOP-10_3x3mm_P0.5mm</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3252,30 +3257,30 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>U2,U18,U19</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>INA226AQDGSRQ1</t>
+          <t>C502477</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>High-Side or Low-Side Measurement, Bi-Directional Current and Power Monitor (0-36V) with I2C Compatible Interface, VSSOP-10</t>
+          <t>3A, Step Down Swift Converter, Adjustable Output Voltage, 5.5-36V Input Voltage, PowerSO-8</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>INA226</t>
+          <t>TPS5430DDA</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>VSSOP-10_3x3mm_P0.5mm</t>
+          <t>TI_SO-PowerPAD-8_ThermalVias</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3295,35 +3300,30 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U4,U5,U6</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>C502477</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>3A, Step Down Swift Converter, Adjustable Output Voltage, 5.5-36V Input Voltage, PowerSO-8</t>
+          <t>C466970</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>TPS5430DDA</t>
+          <t>DB125-3.5-2P-GN-S</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>TI_SO-PowerPAD-8_ThermalVias</t>
+          <t>CONN-TH_2P-P3.50_L7.4-W7.0</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3338,25 +3338,25 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>U4,U5,U6</t>
+          <t>U7,U9,U12,U13</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>C466970</t>
+          <t>C466971</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>DB125-3.5-2P-GN-S</t>
+          <t>DB125-3.5-3P-GN-S</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>CONN-TH_2P-P3.50_L7.4-W7.0</t>
+          <t>CONN-TH_3P-P3.50_L7.4-W10.5</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3376,30 +3376,35 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>U7,U9,U12,U13</t>
+          <t>U8</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>C466971</t>
+          <t>C42417293</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2.4 GHz WiFi (802.11 b/g/n) and Bluetooth ® 5 (LE) module Built around ESP32S3 series of SoCs, Xtensa ® dualcore 32bit LX7 microprocessor Flash up to 16 MB, PSRAM up to 8 MB 36 GPIOs, rich set of peripherals Onboard PCB antenna</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>DB125-3.5-3P-GN-S</t>
+          <t>ESP32-S3-WROOM-2-N32R16V</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>CONN-TH_3P-P3.50_L7.4-W10.5</t>
+          <t>ESP32-S3-WROOM-2</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3414,7 +3419,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -3422,22 +3427,17 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>C42417293</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>2.4 GHz WiFi (802.11 b/g/n) and Bluetooth ® 5 (LE) module Built around ESP32S3 series of SoCs, Xtensa ® dualcore 32bit LX7 microprocessor Flash up to 16 MB, PSRAM up to 8 MB 36 GPIOs, rich set of peripherals Onboard PCB antenna</t>
+          <t>C12084</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-2-N32R16V</t>
+          <t>SN65HVD230DR</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-2</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3457,25 +3457,25 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U14,U16,U17,U21</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>C12084</t>
+          <t>C3008369</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>SN65HVD230DR</t>
+          <t>PC817C-S</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>SOP-4_L6.5-W4.6-P2.54-LS10.3-TL</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -3495,25 +3495,25 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>U14,U16,U17,U21</t>
+          <t>U22</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>C3008369</t>
+          <t>C7835</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>PC817C-S</t>
+          <t>SN74LVC1G14DBVR</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>SOP-4_L6.5-W4.6-P2.54-LS10.3-TL</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>U22</t>
+          <t>U23</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -3541,17 +3541,17 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>C7835</t>
+          <t>C640313</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>SN74LVC1G14DBVR</t>
+          <t>MCP1407-E/MF_C640313</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>DFN-8_L6.0-W5.0-P1.27-BL-EP4.0</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -3571,35 +3571,40 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>U23</t>
+          <t>F1-FUSE</t>
         </is>
       </c>
       <c r="C77" t="n">
         <v>1</v>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Littelfuse</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>C640313</t>
+          <t>0297002.WXNV</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>LOOSE - MINI blade fuse 2A 32V for holder F1 (XF-506P)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>MCP1407-E/MF_C640313</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>DFN-8_L6.0-W5.0-P1.27-BL-EP4.0</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>Top</t>
+          <t>LOOSE</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Supply loose - do NOT mount</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3614,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>F1-FUSE</t>
+          <t>F2-FUSE</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -3622,17 +3627,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0297002.WXNV</t>
+          <t>0297001.WXNV</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>LOOSE - MINI blade fuse 2A 32V for holder F1 (XF-506P)</t>
+          <t>LOOSE - MINI blade fuse 1A 32V for holder F2 (XF-506P)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3652,11 +3657,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>F2-FUSE</t>
+          <t>F3-FUSE,F4-FUSE</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3665,17 +3670,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>0297001.WXNV</t>
+          <t>0297010.WXNV</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>LOOSE - MINI blade fuse 1A 32V for holder F2 (XF-506P)</t>
+          <t>LOOSE - MINI blade fuse 10A 32V for holders F3, F4 (XF-506P)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>10A</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3695,30 +3700,20 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>F3-FUSE,F4-FUSE</t>
+          <t>JP1-SHUNT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2</v>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Littelfuse</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>0297010.WXNV</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>LOOSE - MINI blade fuse 10A 32V for holders F3, F4 (XF-506P)</t>
+          <t>LOOSE - 2-pin 1.27 mm pitch jumper shunt for JP1 (CAN termination; leave JP1 open)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>Jumper 1.27mm</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -3727,39 +3722,6 @@
         </is>
       </c>
       <c r="K80" t="inlineStr">
-        <is>
-          <t>Supply loose - do NOT mount</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>JP1-SHUNT</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>1</v>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>LOOSE - 2-pin 1.27 mm pitch jumper shunt for JP1 (CAN termination; leave JP1 open)</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Jumper 1.27mm</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>LOOSE</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
         <is>
           <t>Supply loose - do NOT mount</t>
         </is>

</xml_diff>

<commit_message>
MarineBoard 1.9.1: routed PCB + fab package rebuilt (#183)
PCB updated from the d7f7e75 schematic and routed (human): D17 buzzer
flyback, D21 D5 VDD diode (bottom), TP1-TP6 test pads, U23 VDD on +12V,
U2 VBUS=Vin+, CAN on GPIO5/6; removed C10/C21-C23/R13.
fab_package.py green: DRC errors 0, unconnected 0, schematic parity 0
(8 silkscreen warnings only). BOM/positions: D17/D21 in, TPs and removed
parts out. Ready for PCBWay re-upload.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MarineBoard/production/MarineBoard-BOM.xlsx
+++ b/MarineBoard/production/MarineBoard-BOM.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K80"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -711,25 +711,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C10,C30</t>
+          <t>C11,C12,C14,C19,C42</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CL05A475MP5NRNC</t>
+          <t>CL05B104KB5NNNC</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4.7uF ±20% 10V Ceramic Capacitor X5R 0402</t>
+          <t>100nF ±10% 50V Ceramic Capacitor X7R 0402</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4.7uF</t>
+          <t>0.1uF</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -754,30 +754,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C11,C12,C14,C19,C42</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CL05B104KB5NNNC</t>
+          <t>GRM21BR61H106KE43L</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>100nF ±10% 50V Ceramic Capacitor X7R 0402</t>
+          <t>10uF ±10% 50V Ceramic Capacitor X5R 0805</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.1uF</t>
+          <t>10uF/50V</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>C_0402_1005Metric</t>
+          <t>C_0805_2012Metric</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -805,22 +805,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GRM21BR61H106KE43L</t>
+          <t>GRM31CR61E476ME44L</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10uF ±10% 50V Ceramic Capacitor X5R 0805</t>
+          <t>47uF ±20% 25V Ceramic Capacitor X5R 1206</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10uF/50V</t>
+          <t>47uF</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>C_0805_2012Metric</t>
+          <t>C_1206_3216Metric</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -848,17 +848,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>GRM31CR61E476ME44L</t>
+          <t>C51205</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>47uF ±20% 25V Ceramic Capacitor X5R 1206</t>
+          <t>4.7uF ±10% 50V Ceramic Capacitor X7R 1206</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>47uF</t>
+          <t>4.7uF</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -891,17 +891,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>C51205</t>
+          <t>C13585</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>4.7uF ±10% 50V Ceramic Capacitor X7R 1206</t>
+          <t>10uF ±10% 50V Ceramic Capacitor X5R 1206</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4.7uF</t>
+          <t>10uF</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -934,22 +934,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>C13585</t>
+          <t>CL05B103KB5NNNC</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10uF ±10% 50V Ceramic Capacitor X5R 1206</t>
+          <t>10nF ±10% 50V Ceramic Capacitor X7R 0402</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10uF</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>C_1206_3216Metric</t>
+          <t>C_0402_1005Metric</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -977,22 +977,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CL05B103KB5NNNC</t>
+          <t>10SVPE220M</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10nF ±10% 50V Ceramic Capacitor X7R 0402</t>
+          <t>220uF ±20% 10V OS-CON polymer, ESR 20mΩ, SMD D6.3xL5.9mm (TPS5430 internal comp needs ESR &lt;=40mΩ)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>220uF 10V</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>C_0402_1005Metric</t>
+          <t>CAP-SMD_BD6.3-L6.6-W6.6-FD</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1012,30 +1012,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C26,C29</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10SVPE220M</t>
+          <t>GCM155R71H473KE02D</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>220uF ±20% 10V OS-CON polymer, ESR 20mΩ, SMD D6.3xL5.9mm (TPS5430 internal comp needs ESR &lt;=40mΩ)</t>
+          <t>47nF ±10% 50V Ceramic Capacitor X7R 0402</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>220uF 10V</t>
+          <t>47nF</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CAP-SMD_BD6.3-L6.6-W6.6-FD</t>
+          <t>C_0402_1005Metric</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -1055,25 +1055,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C26,C29</t>
+          <t>C30</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GCM155R71H473KE02D</t>
+          <t>CL05A475MP5NRNC</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>47nF ±10% 50V Ceramic Capacitor X7R 0402</t>
+          <t>4.7uF ±20% 10V Ceramic Capacitor X5R 0402</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>47nF</t>
+          <t>4.7uF</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>D1,D4,D15</t>
+          <t>D1,D4,D15,D17</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1774,17 +1774,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>C70426</t>
+          <t>1N4148W-7-F</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>75V 150mA switching diode SOD-123; drops D5 VDD ~0.65 V so 3.3 V data meets WS2812B VIH (#183)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>S3MB-13-F</t>
+          <t>1N4148W</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>D_SMB</t>
+          <t>D_SOD-123</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1794,7 +1799,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1809,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1812,22 +1817,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>C492610</t>
+          <t>C70426</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>S3MB-13-F</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>FUSE-TH_XF-506P</t>
+          <t>D_SMB</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1842,7 +1847,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1855,7 +1860,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1880,11 +1885,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>F3,F4</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1893,7 +1898,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1918,35 +1923,30 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Flash1</t>
+          <t>F3,F4</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>C318884</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Push button switch, generic, two pins</t>
+          <t>C492610</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Flash</t>
+          <t>10A</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>SW_Push_1P1T_XKB_TS-1187A</t>
+          <t>FUSE-TH_XF-506P</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>Flash1</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1969,22 +1969,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>C2894897</t>
+          <t>C318884</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>USB 2.0-only 16P Type-C Receptacle connector</t>
+          <t>Push button switch, generic, two pins</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>USB_C_Receptacle_USB2.0_16P</t>
+          <t>Flash</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>USB_C_Receptacle_HCTL_HC-TYPE-C-16P-01A</t>
+          <t>SW_Push_1P1T_XKB_TS-1187A</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>JP1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2012,32 +2012,32 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>C703015</t>
+          <t>C2894897</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>USB 2.0-only 16P Type-C Receptacle connector</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>CAN Bus Term</t>
+          <t>USB_C_Receptacle_USB2.0_16P</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>PinHeader_1x02_P1.27mm_Vertical</t>
+          <t>USB_C_Receptacle_HCTL_HC-TYPE-C-16P-01A</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
           <t>Top</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Leave open - supply shunt loose</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>JP1</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2055,27 +2055,32 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>C435392</t>
+          <t>C703015</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>1uH 3.3A 40mΩ</t>
+          <t>CAN Bus Term</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>L_1008_2520Metric</t>
+          <t>PinHeader_1x02_P1.27mm_Vertical</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
           <t>Top</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Leave open - supply shunt loose</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2090,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2093,17 +2098,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>C5368704</t>
+          <t>C435392</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>22uH</t>
+          <t>1uH 3.3A 40mΩ</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>IND-SMD_L12.5-W12.5_B82477P4XX</t>
+          <t>L_1008_2520Metric</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2113,7 +2118,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2123,35 +2128,25 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>L3,L4,L6</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>muRata(村田)</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>C79382</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>标称阻抗@测试频率:120Ω@100MHz;误差:±25%;直流电阻(RDC):30mΩ;</t>
+          <t>C5368704</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>BLM21PG121SN1D</t>
+          <t>22uH</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>L_0805_2012Metric</t>
+          <t>IND-SMD_L12.5-W12.5_B82477P4XX</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2161,7 +2156,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -2171,25 +2166,35 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>L3,L4,L6</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>muRata(村田)</t>
+        </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>C225048</t>
+          <t>C79382</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>标称阻抗@测试频率:120Ω@100MHz;误差:±25%;直流电阻(RDC):30mΩ;</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>CDRH104RNP-150NC</t>
+          <t>BLM21PG121SN1D</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>IND-SMD_L10.2-W10.0</t>
+          <t>L_0805_2012Metric</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2199,7 +2204,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -2209,25 +2214,25 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>L7,L9,L10</t>
+          <t>L5</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>C74764</t>
+          <t>C225048</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>FerriteBead</t>
+          <t>CDRH104RNP-150NC</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>L_0805_2012Metric</t>
+          <t>IND-SMD_L10.2-W10.0</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2237,7 +2242,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2247,25 +2252,25 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>L8</t>
+          <t>L7,L9,L10</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>C97856</t>
+          <t>C74764</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>DLW21SN900SQ2L</t>
+          <t>FerriteBead</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>FILTER-SMD_4P-L2.0-W1.2-BL_DLW21H</t>
+          <t>L_0805_2012Metric</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2285,35 +2290,25 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Q2,Q3</t>
+          <t>L8</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>宏嘉诚</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>C20069125</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>晶体管类型:NPN;集电极电流(Ic):500mA;集射极击穿电压(Vceo):25V;耗散功率(Pd):300mW;直流电流增益(hFE):120@50mA,1.0V;</t>
+          <t>C97856</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>S8050</t>
+          <t>DLW21SN900SQ2L</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>FILTER-SMD_4P-L2.0-W1.2-BL_DLW21H</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2333,25 +2328,35 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q2,Q3</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>宏嘉诚</t>
+        </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>C52191006</t>
+          <t>C20069125</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>晶体管类型:NPN;集电极电流(Ic):500mA;集射极击穿电压(Vceo):25V;耗散功率(Pd):300mW;直流电流增益(hFE):120@50mA,1.0V;</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>BUK762R4-60E</t>
+          <t>S8050</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TO-263-2_L10.1-W9.1-P5.08-LS15.2-BR</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2361,7 +2366,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -2371,30 +2376,25 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>R1,R2</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>C25905</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C52191006</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>5.1K</t>
+          <t>BUK762R4-60E</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>TO-263-2_L10.1-W9.1-P5.08-LS15.2-BR</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2414,15 +2414,15 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>R3,R10,R15,R20,R25,R26,R27,R28,R32,R40,R42,R43</t>
+          <t>R1,R2</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>5.1K</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -2457,25 +2457,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3,R10,R15,R20,R25,R26,R27,R28,R32,R40,R42,R43</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>C149504</t>
+          <t>C25744</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>100K</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2485,7 +2490,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -2495,30 +2500,25 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>R5,R6</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>C25105</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C149504</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>33R</t>
+          <t>100K</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2538,25 +2538,30 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>R7,R9,R35,R36</t>
+          <t>R5,R6</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>C2907296</t>
+          <t>C25105</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>33R</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2576,25 +2581,20 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R7,R9,R35,R36</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>C17560</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>22KΩ (2202) ±1%</t>
+          <t>C2907296</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>22K</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2627,17 +2627,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>C2089436</t>
+          <t>C17560</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>22KΩ (2202) ±1%</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>200m</t>
+          <t>22K</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>R_0201_0603Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2647,7 +2652,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2662,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -2665,17 +2670,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>C53159429</t>
+          <t>C2089436</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>3k24</t>
+          <t>200m</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_0201_0603Metric</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2685,7 +2690,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -2695,25 +2700,25 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>R14,R19,R21,R23,R24,R49,R50</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>C17437</t>
+          <t>C53159429</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>3k24</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2723,7 +2728,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2733,25 +2738,25 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R14,R19,R21,R23,R24,R49,R50</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>C25718</t>
+          <t>C17437</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>10K/1W</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2761,7 +2766,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -2771,30 +2776,25 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>R22,R29,R30,R41,R44</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>C11702</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C25718</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>10K/1W</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2814,25 +2814,30 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>R31</t>
+          <t>R22,R29,R30,R41,R44</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>C17408</t>
+          <t>C11702</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2842,7 +2847,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2857,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>R33</t>
+          <t>R31</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -2860,22 +2865,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>C25117</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C17408</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>470R</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -2903,22 +2903,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>0402WGF1000TCE</t>
+          <t>C25117</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>100Ω (1000) ±1%</t>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>470R</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -2938,25 +2938,30 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>R38,R39</t>
+          <t>R34</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>C48996903</t>
+          <t>0402WGF1000TCE</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>100Ω (1000) ±1%</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R0402</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -2966,7 +2971,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -2976,25 +2981,25 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>R46</t>
+          <t>R38,R39</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>C175364</t>
+          <t>C48996903</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>47K/1W</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0805_2012Metric</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3004,7 +3009,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3019,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>R47</t>
+          <t>R46</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -3022,12 +3027,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>C2075262</t>
+          <t>C175364</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2K2</t>
+          <t>47K/1W</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3042,7 +3047,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3057,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>R47</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -3060,22 +3065,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>C25792</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+          <t>C2075262</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>47K</t>
+          <t>2K2</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>R_0402_1005Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Relay1</t>
+          <t>R48</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -3103,22 +3103,27 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>C30431</t>
+          <t>C25792</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>SRD-12VDC-SL-C</t>
+          <t>47K</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>RELAY-TH_SRD-XXVDC-XL-C</t>
+          <t>R_0402_1005Metric</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3133,7 +3138,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Reset1</t>
+          <t>Relay1</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -3141,27 +3146,22 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>C318884</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Push button switch, generic, two pins</t>
+          <t>C30431</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Reset</t>
+          <t>SRD-12VDC-SL-C</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>SW_Push_1P1T_XKB_TS-1187A</t>
+          <t>RELAY-TH_SRD-XXVDC-XL-C</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>Reset1</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -3184,17 +3184,22 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>C479074</t>
+          <t>C318884</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Push button switch, generic, two pins</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>SY8089A1AAC</t>
+          <t>Reset</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>TSOT-23-5</t>
+          <t>SW_Push_1P1T_XKB_TS-1187A</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3214,30 +3219,25 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>U2,U18,U19</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>INA226AQDGSRQ1</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>High-Side or Low-Side Measurement, Bi-Directional Current and Power Monitor (0-36V) with I2C Compatible Interface, VSSOP-10</t>
+          <t>C479074</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>INA226</t>
+          <t>SY8089A1AAC</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>VSSOP-10_3x3mm_P0.5mm</t>
+          <t>TSOT-23-5</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3257,30 +3257,30 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2,U18,U19</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>C502477</t>
+          <t>INA226AQDGSRQ1</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>3A, Step Down Swift Converter, Adjustable Output Voltage, 5.5-36V Input Voltage, PowerSO-8</t>
+          <t>High-Side or Low-Side Measurement, Bi-Directional Current and Power Monitor (0-36V) with I2C Compatible Interface, VSSOP-10</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>TPS5430DDA</t>
+          <t>INA226</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>TI_SO-PowerPAD-8_ThermalVias</t>
+          <t>VSSOP-10_3x3mm_P0.5mm</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3300,30 +3300,35 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>U4,U5,U6</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>C466970</t>
+          <t>C502477</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>3A, Step Down Swift Converter, Adjustable Output Voltage, 5.5-36V Input Voltage, PowerSO-8</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>DB125-3.5-2P-GN-S</t>
+          <t>TPS5430DDA</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>CONN-TH_2P-P3.50_L7.4-W7.0</t>
+          <t>TI_SO-PowerPAD-8_ThermalVias</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3338,25 +3343,25 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>U7,U9,U12,U13</t>
+          <t>U4,U5,U6</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>C466971</t>
+          <t>C466970</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>DB125-3.5-3P-GN-S</t>
+          <t>DB125-3.5-2P-GN-S</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>CONN-TH_3P-P3.50_L7.4-W10.5</t>
+          <t>CONN-TH_2P-P3.50_L7.4-W7.0</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3376,35 +3381,30 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U7,U9,U12,U13</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>C42417293</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>2.4 GHz WiFi (802.11 b/g/n) and Bluetooth ® 5 (LE) module Built around ESP32S3 series of SoCs, Xtensa ® dualcore 32bit LX7 microprocessor Flash up to 16 MB, PSRAM up to 8 MB 36 GPIOs, rich set of peripherals Onboard PCB antenna</t>
+          <t>C466971</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-2-N32R16V</t>
+          <t>DB125-3.5-3P-GN-S</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-2</t>
+          <t>CONN-TH_3P-P3.50_L7.4-W10.5</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U8</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -3427,17 +3427,22 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>C12084</t>
+          <t>C42417293</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2.4 GHz WiFi (802.11 b/g/n) and Bluetooth ® 5 (LE) module Built around ESP32S3 series of SoCs, Xtensa ® dualcore 32bit LX7 microprocessor Flash up to 16 MB, PSRAM up to 8 MB 36 GPIOs, rich set of peripherals Onboard PCB antenna</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>SN65HVD230DR</t>
+          <t>ESP32-S3-WROOM-2-N32R16V</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>ESP32-S3-WROOM-2</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3457,25 +3462,25 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>U14,U16,U17,U21</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>C3008369</t>
+          <t>C12084</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>PC817C-S</t>
+          <t>SN65HVD230DR</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>SOP-4_L6.5-W4.6-P2.54-LS10.3-TL</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3485,7 +3490,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Bottom/Top</t>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -3495,25 +3500,25 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>U22</t>
+          <t>U14,U16,U17,U21</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>C7835</t>
+          <t>C3008369</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>SN74LVC1G14DBVR</t>
+          <t>PC817C-S</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>SOP-4_L6.5-W4.6-P2.54-LS10.3-TL</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3523,7 +3528,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Bottom/Top</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3538,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>U23</t>
+          <t>U22</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -3541,17 +3546,17 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>C640313</t>
+          <t>C7835</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>MCP1407-E/MF_C640313</t>
+          <t>SN74LVC1G14DBVR</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>DFN-8_L6.0-W5.0-P1.27-BL-EP4.0</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3561,7 +3566,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
     </row>
@@ -3571,40 +3576,35 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>F1-FUSE</t>
+          <t>U23</t>
         </is>
       </c>
       <c r="C77" t="n">
         <v>1</v>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Littelfuse</t>
-        </is>
-      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>0297002.WXNV</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>LOOSE - MINI blade fuse 2A 32V for holder F1 (XF-506P)</t>
+          <t>C640313</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2A</t>
+          <t>MCP1407-E/MF_C640313</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>DFN-8_L6.0-W5.0-P1.27-BL-EP4.0</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>LOOSE</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>Supply loose - do NOT mount</t>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Top</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>F2-FUSE</t>
+          <t>F1-FUSE</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -3627,17 +3627,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0297001.WXNV</t>
+          <t>0297002.WXNV</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>LOOSE - MINI blade fuse 1A 32V for holder F2 (XF-506P)</t>
+          <t>LOOSE - MINI blade fuse 2A 32V for holder F1 (XF-506P)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>1A</t>
+          <t>2A</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3657,11 +3657,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>F3-FUSE,F4-FUSE</t>
+          <t>F2-FUSE</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3670,17 +3670,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>0297010.WXNV</t>
+          <t>0297001.WXNV</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>LOOSE - MINI blade fuse 10A 32V for holders F3, F4 (XF-506P)</t>
+          <t>LOOSE - MINI blade fuse 1A 32V for holder F2 (XF-506P)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>10A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3700,28 +3700,71 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
+          <t>F3-FUSE,F4-FUSE</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Littelfuse</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0297010.WXNV</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>LOOSE - MINI blade fuse 10A 32V for holders F3, F4 (XF-506P)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>LOOSE</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Supply loose - do NOT mount</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>JP1-SHUNT</t>
         </is>
       </c>
-      <c r="C80" t="n">
-        <v>1</v>
-      </c>
-      <c r="F80" t="inlineStr">
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="inlineStr">
         <is>
           <t>LOOSE - 2-pin 1.27 mm pitch jumper shunt for JP1 (CAN termination; leave JP1 open)</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>Jumper 1.27mm</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
+      <c r="I81" t="inlineStr">
         <is>
           <t>LOOSE</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr">
+      <c r="K81" t="inlineStr">
         <is>
           <t>Supply loose - do NOT mount</t>
         </is>

</xml_diff>